<commit_message>
Updated for PR feedback
</commit_message>
<xml_diff>
--- a/rules/CORE-000594/negative/01/data/unit-test-coreid-CG0359-negative.xlsx
+++ b/rules/CORE-000594/negative/01/data/unit-test-coreid-CG0359-negative.xlsx
@@ -36,7 +36,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" mc:Ignorable="x14ac">
   <numFmts count="0"/>
-  <fonts count="5" x14ac:knownFonts="1">
+  <fonts count="6" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <name val="Calibri"/>
@@ -59,8 +59,13 @@
       <name val="Calibri"/>
       <i/>
     </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+      <i/>
+    </font>
   </fonts>
-  <fills count="3">
+  <fills count="4">
     <fill>
       <patternFill patternType="none">
         <bgColor/>
@@ -68,6 +73,12 @@
     </fill>
     <fill>
       <patternFill patternType="gray125">
+        <bgColor/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFFCC"/>
         <bgColor/>
       </patternFill>
     </fill>
@@ -97,13 +108,14 @@
   <cellStyleXfs>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="1" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
   </cellXfs>
   <cellStyles>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -548,7 +560,7 @@
         <v>variable_label</v>
       </c>
       <c r="F3" s="4" t="str">
-        <v>domain abbreviation</v>
+        <v>domain Abbreviation</v>
       </c>
     </row>
     <row r="4">
@@ -606,59 +618,59 @@
       <c r="A2" s="5" t="str">
         <v>study identifier</v>
       </c>
-      <c r="B2" s="5" t="str">
-        <v>domain abbreviation</v>
-      </c>
-      <c r="C2" s="5" t="str">
+      <c r="B2" s="6" t="str">
+        <v>domain Abbreviation</v>
+      </c>
+      <c r="C2" s="6" t="str">
         <v>unique subject identifier</v>
       </c>
-      <c r="D2" s="5" t="str">
+      <c r="D2" s="6" t="str">
         <v>Serious Event 1</v>
       </c>
-      <c r="E2" s="5" t="str">
+      <c r="E2" s="6" t="str">
         <v>A1ction Taken With Study Treatment</v>
       </c>
-      <c r="F2" s="5" t="str">
+      <c r="F2" s="6" t="str">
         <v>Causality $</v>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="5" t="str">
+      <c r="A3" s="6" t="str">
         <v>Char</v>
       </c>
-      <c r="B3" s="5" t="str">
+      <c r="B3" s="6" t="str">
         <v>Char</v>
       </c>
-      <c r="C3" s="5" t="str">
+      <c r="C3" s="6" t="str">
         <v>Char</v>
       </c>
-      <c r="D3" s="5" t="str">
+      <c r="D3" s="6" t="str">
         <v>Char</v>
       </c>
-      <c r="E3" s="5" t="str">
+      <c r="E3" s="6" t="str">
         <v>Char</v>
       </c>
-      <c r="F3" s="5" t="str">
+      <c r="F3" s="6" t="str">
         <v>Char</v>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="5">
+      <c r="A4" s="6">
         <v>10</v>
       </c>
-      <c r="B4" s="5">
+      <c r="B4" s="6">
         <v>2</v>
       </c>
-      <c r="C4" s="5">
+      <c r="C4" s="6">
         <v>14</v>
       </c>
-      <c r="D4" s="5">
+      <c r="D4" s="6">
         <v>1</v>
       </c>
-      <c r="E4" s="5">
+      <c r="E4" s="6">
         <v>1</v>
       </c>
-      <c r="F4" s="5">
+      <c r="F4" s="6">
         <v>1</v>
       </c>
     </row>

</xml_diff>